<commit_message>
fix: enforce metric consistency across README, app, Word report, and Basel III Excel schedule
</commit_message>
<xml_diff>
--- a/excel/CreditLens_Portfolio_Model.xlsx
+++ b/excel/CreditLens_Portfolio_Model.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Executive_Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Loan_Tape_Sample" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Model_Diagnostics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive_Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loan_Tape_Sample" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Diagnostics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECL_Schedule" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,8 +82,13 @@
       <i val="1"/>
       <color rgb="006B7280"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -113,8 +119,14 @@
         <bgColor rgb="000F172A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+        <bgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -136,11 +148,25 @@
         <color rgb="00D1D5DB"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="001E3A8A"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001E3A8A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -187,6 +213,13 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="10" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -25521,4 +25554,510 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="106" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>BASEL III / IFRS 9 EXPECTED CREDIT LOSS (ECL) RESERVE SCHEDULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Standardized Framework: ECL = EAD × PD × LGD | Standard LGD = 45.0% | CCF = 20.0% (Undrawn Commitments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>1. FULL PORTFOLIO CAPITAL RESERVES (30,000 ACCOUNTS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Risk Tier</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Borrowers</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Portfolio Share %</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Total Credit Line (NTD)</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Drawn Balance (NTD)</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Exposure at Default (EAD)</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>Average PD %</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>LGD %</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>ECL Reserve (NTD)</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>ECL Coverage %</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Prime</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>8050</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>0.2683</v>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>2025000000</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>528349269</v>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>827739330.4</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>0.1696</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>61885866.6</v>
+      </c>
+      <c r="K7" s="12" t="n">
+        <v>0.07480000000000001</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Near-Prime</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>7558</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>0.2519</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>1296680000</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>433389146</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>607877285</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>0.2912</v>
+      </c>
+      <c r="I8" s="16" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J8" s="17" t="n">
+        <v>78818378.40000001</v>
+      </c>
+      <c r="K8" s="16" t="n">
+        <v>0.1297</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Subprime</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>6507</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>0.2169</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>823983680</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>248387028</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>365105928.2</v>
+      </c>
+      <c r="H9" s="12" t="n">
+        <v>0.4079</v>
+      </c>
+      <c r="I9" s="12" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J9" s="13" t="n">
+        <v>66426404.8</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>0.1819</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>7885</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>0.2628</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>878866000</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>326574484</v>
+      </c>
+      <c r="G10" s="17" t="n">
+        <v>438686701.2</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>0.7169</v>
+      </c>
+      <c r="I10" s="16" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J10" s="17" t="n">
+        <v>145021826.6</v>
+      </c>
+      <c r="K10" s="16" t="n">
+        <v>0.3306</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>Total Portfolio</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D11" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <v>5024529680</v>
+      </c>
+      <c r="F11" s="30" t="n">
+        <v>1536699927</v>
+      </c>
+      <c r="G11" s="30" t="n">
+        <v>2239409244.8</v>
+      </c>
+      <c r="H11" s="29" t="n">
+        <v>0.3494</v>
+      </c>
+      <c r="I11" s="29" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J11" s="30" t="n">
+        <v>352152476.4</v>
+      </c>
+      <c r="K11" s="29" t="n">
+        <v>0.1573</v>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14">
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>2. HOLDOUT VALIDATION SET CAPITAL RESERVES (6,000 UNSEEN ACCOUNTS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Risk Tier</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Borrowers</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Portfolio Share %</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Total Credit Line (NTD)</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Drawn Balance (NTD)</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Exposure at Default (EAD)</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Average PD %</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>LGD %</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>ECL Reserve (NTD)</t>
+        </is>
+      </c>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>ECL Coverage %</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Prime</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>1558</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>0.2597</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>395430000</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>101343637</v>
+      </c>
+      <c r="G16" s="17" t="n">
+        <v>160168618.4</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <v>0.1704</v>
+      </c>
+      <c r="I16" s="16" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J16" s="17" t="n">
+        <v>11956757.6</v>
+      </c>
+      <c r="K16" s="16" t="n">
+        <v>0.0747</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Near-Prime</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>1563</v>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>0.2605</v>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>275840000</v>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>90369323</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>127768575.6</v>
+      </c>
+      <c r="H17" s="12" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="I17" s="12" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J17" s="13" t="n">
+        <v>16590225.7</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>0.1298</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Subprime</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="n">
+        <v>1323</v>
+      </c>
+      <c r="D18" s="16" t="n">
+        <v>0.2205</v>
+      </c>
+      <c r="E18" s="17" t="n">
+        <v>164167680</v>
+      </c>
+      <c r="F18" s="17" t="n">
+        <v>51197287</v>
+      </c>
+      <c r="G18" s="17" t="n">
+        <v>74239639.59999999</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <v>0.4074</v>
+      </c>
+      <c r="I18" s="16" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J18" s="17" t="n">
+        <v>13503597.6</v>
+      </c>
+      <c r="K18" s="16" t="n">
+        <v>0.1819</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>1556</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>0.2593</v>
+      </c>
+      <c r="E19" s="13" t="n">
+        <v>172340000</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>67377626</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>88718395.40000001</v>
+      </c>
+      <c r="H19" s="12" t="n">
+        <v>0.7153</v>
+      </c>
+      <c r="I19" s="12" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J19" s="13" t="n">
+        <v>29384122.6</v>
+      </c>
+      <c r="K19" s="12" t="n">
+        <v>0.3312</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>Total Holdout (Unseen)</t>
+        </is>
+      </c>
+      <c r="C20" s="28" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D20" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="30" t="n">
+        <v>1007777680</v>
+      </c>
+      <c r="F20" s="30" t="n">
+        <v>310287873</v>
+      </c>
+      <c r="G20" s="30" t="n">
+        <v>450895229</v>
+      </c>
+      <c r="H20" s="29" t="n">
+        <v>0.3521</v>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J20" s="30" t="n">
+        <v>71434703.5</v>
+      </c>
+      <c r="K20" s="29" t="n">
+        <v>0.1584</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:K2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>